<commit_message>
Completar planilla y normalizar guía EVA 1
</commit_message>
<xml_diff>
--- a/FASE 1/EVIDENCIAS_GRUPALES/PLANILLA DE EVALUACIÓN FASE 1.xlsx
+++ b/FASE 1/EVIDENCIAS_GRUPALES/PLANILLA DE EVALUACIÓN FASE 1.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="98">
   <si>
     <t>INTEGRANTES</t>
   </si>
@@ -378,6 +378,15 @@
   </si>
   <si>
     <t>Muy Relevante</t>
+  </si>
+  <si>
+    <t>Felipe Arce</t>
+  </si>
+  <si>
+    <t>Daniel Baeza</t>
+  </si>
+  <si>
+    <t>Benjamín Olmedo</t>
   </si>
 </sst>
 </file>
@@ -1481,7 +1490,9 @@
       <c r="A4" s="5">
         <v>1</v>
       </c>
-      <c r="B4" s="32"/>
+      <c r="B4" s="32" t="s">
+        <v>95</v>
+      </c>
       <c r="C4" s="6">
         <f>EVALUACION1!$C$24</f>
         <v>7</v>
@@ -1500,7 +1511,9 @@
       <c r="A5" s="5">
         <v>2</v>
       </c>
-      <c r="B5" s="32"/>
+      <c r="B5" s="32" t="s">
+        <v>96</v>
+      </c>
       <c r="C5" s="6">
         <f>EVALUACION1!$C$24</f>
         <v>7</v>
@@ -1519,7 +1532,9 @@
       <c r="A6" s="5">
         <v>3</v>
       </c>
-      <c r="B6" s="32"/>
+      <c r="B6" s="32" t="s">
+        <v>97</v>
+      </c>
       <c r="C6" s="6">
         <f>EVALUACION1!$C$24</f>
         <v>7</v>
@@ -2046,9 +2061,9 @@
       <c r="B27" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="52">
+      <c r="C27" s="52" t="str">
         <f>$B$4</f>
-        <v>0</v>
+        <v>Felipe Arce</v>
       </c>
       <c r="D27" s="53"/>
       <c r="E27" s="53"/>
@@ -2296,9 +2311,9 @@
       <c r="B39" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C39" s="52">
+      <c r="C39" s="52" t="str">
         <f>B5</f>
-        <v>0</v>
+        <v>Daniel Baeza</v>
       </c>
       <c r="D39" s="53"/>
       <c r="E39" s="53"/>
@@ -2545,9 +2560,9 @@
       <c r="B50" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="52">
+      <c r="C50" s="52" t="str">
         <f>B6</f>
-        <v>0</v>
+        <v>Benjamín Olmedo</v>
       </c>
       <c r="D50" s="53"/>
       <c r="E50" s="53"/>

</xml_diff>